<commit_message>
Fix initializeDefaultAttendanceForClass bug causing UI freeze on class change, and update Excel data
</commit_message>
<xml_diff>
--- a/TBTA-2026-2027- RHS-Student_Attendance.xlsx
+++ b/TBTA-2026-2027- RHS-Student_Attendance.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maniv\all_ide_code_ws\apps\attendance-tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCF5E77-5D5B-41BF-976C-F11FF5D38083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD757AD-9959-4FA6-8646-BA1536737575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FHS" sheetId="2" state="hidden" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3206" uniqueCount="762">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3201" uniqueCount="761">
   <si>
     <t>First Name</t>
   </si>
@@ -2190,9 +2190,6 @@
   </si>
   <si>
     <t>Saravana Aniruthan</t>
-  </si>
-  <si>
-    <t>Balakrishnan</t>
   </si>
   <si>
     <t>Dhyaan</t>
@@ -2557,7 +2554,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="8">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -2638,11 +2635,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -2901,9 +2926,6 @@
     </xf>
     <xf numFmtId="14" fontId="6" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="9" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="10" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2942,6 +2964,16 @@
     <xf numFmtId="0" fontId="23" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="10" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2991,7 +3023,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:D29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table_1" displayName="Table_1" ref="A1:D28">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Name"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nilai"/>
@@ -10418,7 +10450,7 @@
     </row>
     <row r="226" spans="1:10" ht="14.25" customHeight="1">
       <c r="A226" s="1" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="B226" s="1" t="s">
         <v>35</v>
@@ -10450,7 +10482,7 @@
     </row>
     <row r="227" spans="1:10" ht="14.25" customHeight="1">
       <c r="A227" s="1" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="B227" s="1" t="s">
         <v>577</v>
@@ -10485,7 +10517,7 @@
         <v>103</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="C228" s="2">
         <v>43790</v>
@@ -10514,10 +10546,10 @@
     </row>
     <row r="229" spans="1:10" ht="14.25" customHeight="1">
       <c r="A229" s="1" t="s">
+        <v>720</v>
+      </c>
+      <c r="B229" s="1" t="s">
         <v>721</v>
-      </c>
-      <c r="B229" s="1" t="s">
-        <v>722</v>
       </c>
       <c r="C229" s="2">
         <v>42911</v>
@@ -10578,10 +10610,10 @@
     </row>
     <row r="231" spans="1:10" ht="14.25" customHeight="1">
       <c r="A231" s="1" t="s">
+        <v>723</v>
+      </c>
+      <c r="B231" s="1" t="s">
         <v>724</v>
-      </c>
-      <c r="B231" s="1" t="s">
-        <v>725</v>
       </c>
       <c r="C231" s="2">
         <v>43549</v>
@@ -10610,10 +10642,10 @@
     </row>
     <row r="232" spans="1:10" ht="14.25" customHeight="1">
       <c r="A232" s="1" t="s">
+        <v>725</v>
+      </c>
+      <c r="B232" s="1" t="s">
         <v>726</v>
-      </c>
-      <c r="B232" s="1" t="s">
-        <v>727</v>
       </c>
       <c r="C232" s="2">
         <v>41160</v>
@@ -10642,10 +10674,10 @@
     </row>
     <row r="233" spans="1:10" ht="14.25" customHeight="1">
       <c r="A233" s="1" t="s">
+        <v>727</v>
+      </c>
+      <c r="B233" s="1" t="s">
         <v>728</v>
-      </c>
-      <c r="B233" s="1" t="s">
-        <v>729</v>
       </c>
       <c r="C233" s="2">
         <v>43829</v>
@@ -10674,7 +10706,7 @@
     </row>
     <row r="234" spans="1:10" ht="14.25" customHeight="1">
       <c r="A234" s="1" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="B234" s="1" t="s">
         <v>555</v>
@@ -10706,7 +10738,7 @@
     </row>
     <row r="235" spans="1:10" ht="14.25" customHeight="1">
       <c r="A235" s="1" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="B235" s="1" t="s">
         <v>215</v>
@@ -10738,7 +10770,7 @@
     </row>
     <row r="236" spans="1:10" ht="14.25" customHeight="1">
       <c r="A236" s="1" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B236" s="1" t="s">
         <v>449</v>
@@ -10770,10 +10802,10 @@
     </row>
     <row r="237" spans="1:10" ht="14.25" customHeight="1">
       <c r="A237" s="47" t="s">
+        <v>732</v>
+      </c>
+      <c r="B237" s="47" t="s">
         <v>733</v>
-      </c>
-      <c r="B237" s="47" t="s">
-        <v>734</v>
       </c>
       <c r="C237" s="48">
         <v>42156</v>
@@ -10799,10 +10831,10 @@
     </row>
     <row r="238" spans="1:10" ht="14.25" customHeight="1">
       <c r="A238" s="47" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="B238" s="47" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C238" s="48">
         <v>44145</v>
@@ -10828,12 +10860,12 @@
     </row>
     <row r="239" spans="1:10" ht="14.25" customHeight="1">
       <c r="A239" s="83" t="s">
+        <v>737</v>
+      </c>
+      <c r="B239" s="83" t="s">
         <v>738</v>
       </c>
-      <c r="B239" s="83" t="s">
-        <v>739</v>
-      </c>
-      <c r="C239" s="132">
+      <c r="C239" s="129">
         <v>42825</v>
       </c>
       <c r="D239" s="44" t="s">
@@ -10856,16 +10888,16 @@
       </c>
     </row>
     <row r="240" spans="1:10" ht="14.25" customHeight="1">
-      <c r="A240" s="133" t="s">
+      <c r="A240" s="130" t="s">
+        <v>739</v>
+      </c>
+      <c r="B240" s="130" t="s">
         <v>740</v>
       </c>
-      <c r="B240" s="133" t="s">
-        <v>741</v>
-      </c>
-      <c r="C240" s="134">
+      <c r="C240" s="131">
         <v>41822</v>
       </c>
-      <c r="D240" s="133" t="s">
+      <c r="D240" s="130" t="s">
         <v>28</v>
       </c>
       <c r="E240" s="1" t="s">
@@ -10886,12 +10918,12 @@
     </row>
     <row r="241" spans="1:127" ht="14.25" customHeight="1">
       <c r="A241" s="83" t="s">
+        <v>741</v>
+      </c>
+      <c r="B241" s="83" t="s">
         <v>742</v>
       </c>
-      <c r="B241" s="83" t="s">
-        <v>743</v>
-      </c>
-      <c r="C241" s="135">
+      <c r="C241" s="132">
         <v>42752</v>
       </c>
       <c r="D241" s="83" t="s">
@@ -10912,123 +10944,123 @@
       <c r="J241" s="45">
         <v>46199</v>
       </c>
-      <c r="K241" s="136"/>
-      <c r="L241" s="136"/>
-      <c r="M241" s="136"/>
-      <c r="N241" s="136"/>
-      <c r="O241" s="136"/>
-      <c r="P241" s="136"/>
-      <c r="Q241" s="136"/>
-      <c r="R241" s="136"/>
-      <c r="S241" s="136"/>
-      <c r="T241" s="136"/>
-      <c r="U241" s="136"/>
-      <c r="V241" s="136"/>
-      <c r="W241" s="136"/>
-      <c r="X241" s="136"/>
-      <c r="Y241" s="136"/>
-      <c r="Z241" s="136"/>
-      <c r="AA241" s="136"/>
-      <c r="AB241" s="136"/>
-      <c r="AC241" s="136"/>
-      <c r="AD241" s="136"/>
-      <c r="AE241" s="136"/>
-      <c r="AF241" s="136"/>
-      <c r="AG241" s="136"/>
-      <c r="AH241" s="136"/>
-      <c r="AI241" s="136"/>
-      <c r="AJ241" s="136"/>
-      <c r="AK241" s="136"/>
-      <c r="AL241" s="136"/>
-      <c r="AM241" s="136"/>
-      <c r="AN241" s="136"/>
-      <c r="AO241" s="136"/>
-      <c r="AP241" s="136"/>
-      <c r="AQ241" s="136"/>
-      <c r="AR241" s="136"/>
-      <c r="AS241" s="136"/>
-      <c r="AT241" s="136"/>
-      <c r="AU241" s="136"/>
-      <c r="AV241" s="136"/>
-      <c r="AW241" s="136"/>
-      <c r="AX241" s="136"/>
-      <c r="AY241" s="136"/>
-      <c r="AZ241" s="136"/>
-      <c r="BA241" s="136"/>
-      <c r="BB241" s="136"/>
-      <c r="BC241" s="136"/>
-      <c r="BD241" s="136"/>
-      <c r="BE241" s="136"/>
-      <c r="BF241" s="136"/>
-      <c r="BG241" s="136"/>
-      <c r="BH241" s="136"/>
-      <c r="BI241" s="136"/>
-      <c r="BJ241" s="136"/>
-      <c r="BK241" s="136"/>
-      <c r="BL241" s="136"/>
-      <c r="BM241" s="136"/>
-      <c r="BN241" s="136"/>
-      <c r="BO241" s="136"/>
-      <c r="BP241" s="136"/>
-      <c r="BQ241" s="136"/>
-      <c r="BR241" s="136"/>
-      <c r="BS241" s="136"/>
-      <c r="BT241" s="136"/>
-      <c r="BU241" s="136"/>
-      <c r="BV241" s="136"/>
-      <c r="BW241" s="136"/>
-      <c r="BX241" s="136"/>
-      <c r="BY241" s="136"/>
-      <c r="BZ241" s="136"/>
-      <c r="CA241" s="136"/>
-      <c r="CB241" s="136"/>
-      <c r="CC241" s="136"/>
-      <c r="CD241" s="136"/>
-      <c r="CE241" s="136"/>
-      <c r="CF241" s="136"/>
-      <c r="CG241" s="136"/>
-      <c r="CH241" s="136"/>
-      <c r="CI241" s="136"/>
-      <c r="CJ241" s="136"/>
-      <c r="CK241" s="136"/>
-      <c r="CL241" s="136"/>
-      <c r="CM241" s="136"/>
-      <c r="CN241" s="136"/>
-      <c r="CO241" s="136"/>
-      <c r="CP241" s="136"/>
-      <c r="CQ241" s="136"/>
-      <c r="CR241" s="136"/>
-      <c r="CS241" s="136"/>
-      <c r="CT241" s="136"/>
-      <c r="CU241" s="136"/>
-      <c r="CV241" s="136"/>
-      <c r="CW241" s="136"/>
-      <c r="CX241" s="136"/>
-      <c r="CY241" s="136"/>
-      <c r="CZ241" s="136"/>
-      <c r="DA241" s="136"/>
-      <c r="DB241" s="136"/>
-      <c r="DC241" s="136"/>
-      <c r="DD241" s="136"/>
-      <c r="DE241" s="136"/>
-      <c r="DF241" s="136"/>
-      <c r="DG241" s="136"/>
-      <c r="DH241" s="136"/>
-      <c r="DI241" s="136"/>
-      <c r="DJ241" s="136"/>
-      <c r="DK241" s="136"/>
-      <c r="DL241" s="136"/>
-      <c r="DM241" s="136"/>
-      <c r="DN241" s="136"/>
-      <c r="DO241" s="136"/>
-      <c r="DP241" s="136"/>
-      <c r="DQ241" s="136"/>
-      <c r="DR241" s="136"/>
-      <c r="DS241" s="136"/>
-      <c r="DT241" s="136"/>
-      <c r="DU241" s="136"/>
-      <c r="DV241" s="136"/>
-      <c r="DW241" s="136"/>
+      <c r="K241" s="133"/>
+      <c r="L241" s="133"/>
+      <c r="M241" s="133"/>
+      <c r="N241" s="133"/>
+      <c r="O241" s="133"/>
+      <c r="P241" s="133"/>
+      <c r="Q241" s="133"/>
+      <c r="R241" s="133"/>
+      <c r="S241" s="133"/>
+      <c r="T241" s="133"/>
+      <c r="U241" s="133"/>
+      <c r="V241" s="133"/>
+      <c r="W241" s="133"/>
+      <c r="X241" s="133"/>
+      <c r="Y241" s="133"/>
+      <c r="Z241" s="133"/>
+      <c r="AA241" s="133"/>
+      <c r="AB241" s="133"/>
+      <c r="AC241" s="133"/>
+      <c r="AD241" s="133"/>
+      <c r="AE241" s="133"/>
+      <c r="AF241" s="133"/>
+      <c r="AG241" s="133"/>
+      <c r="AH241" s="133"/>
+      <c r="AI241" s="133"/>
+      <c r="AJ241" s="133"/>
+      <c r="AK241" s="133"/>
+      <c r="AL241" s="133"/>
+      <c r="AM241" s="133"/>
+      <c r="AN241" s="133"/>
+      <c r="AO241" s="133"/>
+      <c r="AP241" s="133"/>
+      <c r="AQ241" s="133"/>
+      <c r="AR241" s="133"/>
+      <c r="AS241" s="133"/>
+      <c r="AT241" s="133"/>
+      <c r="AU241" s="133"/>
+      <c r="AV241" s="133"/>
+      <c r="AW241" s="133"/>
+      <c r="AX241" s="133"/>
+      <c r="AY241" s="133"/>
+      <c r="AZ241" s="133"/>
+      <c r="BA241" s="133"/>
+      <c r="BB241" s="133"/>
+      <c r="BC241" s="133"/>
+      <c r="BD241" s="133"/>
+      <c r="BE241" s="133"/>
+      <c r="BF241" s="133"/>
+      <c r="BG241" s="133"/>
+      <c r="BH241" s="133"/>
+      <c r="BI241" s="133"/>
+      <c r="BJ241" s="133"/>
+      <c r="BK241" s="133"/>
+      <c r="BL241" s="133"/>
+      <c r="BM241" s="133"/>
+      <c r="BN241" s="133"/>
+      <c r="BO241" s="133"/>
+      <c r="BP241" s="133"/>
+      <c r="BQ241" s="133"/>
+      <c r="BR241" s="133"/>
+      <c r="BS241" s="133"/>
+      <c r="BT241" s="133"/>
+      <c r="BU241" s="133"/>
+      <c r="BV241" s="133"/>
+      <c r="BW241" s="133"/>
+      <c r="BX241" s="133"/>
+      <c r="BY241" s="133"/>
+      <c r="BZ241" s="133"/>
+      <c r="CA241" s="133"/>
+      <c r="CB241" s="133"/>
+      <c r="CC241" s="133"/>
+      <c r="CD241" s="133"/>
+      <c r="CE241" s="133"/>
+      <c r="CF241" s="133"/>
+      <c r="CG241" s="133"/>
+      <c r="CH241" s="133"/>
+      <c r="CI241" s="133"/>
+      <c r="CJ241" s="133"/>
+      <c r="CK241" s="133"/>
+      <c r="CL241" s="133"/>
+      <c r="CM241" s="133"/>
+      <c r="CN241" s="133"/>
+      <c r="CO241" s="133"/>
+      <c r="CP241" s="133"/>
+      <c r="CQ241" s="133"/>
+      <c r="CR241" s="133"/>
+      <c r="CS241" s="133"/>
+      <c r="CT241" s="133"/>
+      <c r="CU241" s="133"/>
+      <c r="CV241" s="133"/>
+      <c r="CW241" s="133"/>
+      <c r="CX241" s="133"/>
+      <c r="CY241" s="133"/>
+      <c r="CZ241" s="133"/>
+      <c r="DA241" s="133"/>
+      <c r="DB241" s="133"/>
+      <c r="DC241" s="133"/>
+      <c r="DD241" s="133"/>
+      <c r="DE241" s="133"/>
+      <c r="DF241" s="133"/>
+      <c r="DG241" s="133"/>
+      <c r="DH241" s="133"/>
+      <c r="DI241" s="133"/>
+      <c r="DJ241" s="133"/>
+      <c r="DK241" s="133"/>
+      <c r="DL241" s="133"/>
+      <c r="DM241" s="133"/>
+      <c r="DN241" s="133"/>
+      <c r="DO241" s="133"/>
+      <c r="DP241" s="133"/>
+      <c r="DQ241" s="133"/>
+      <c r="DR241" s="133"/>
+      <c r="DS241" s="133"/>
+      <c r="DT241" s="133"/>
+      <c r="DU241" s="133"/>
+      <c r="DV241" s="133"/>
+      <c r="DW241" s="133"/>
     </row>
     <row r="242" spans="1:127" ht="14.25" customHeight="1"/>
     <row r="243" spans="1:127" ht="14.25" customHeight="1"/>
@@ -12210,10 +12242,10 @@
     </row>
     <row r="15" spans="1:18" ht="14">
       <c r="A15" s="50" t="s">
+        <v>718</v>
+      </c>
+      <c r="B15" s="50" t="s">
         <v>719</v>
-      </c>
-      <c r="B15" s="50" t="s">
-        <v>720</v>
       </c>
       <c r="C15" s="71">
         <v>46090</v>
@@ -12242,14 +12274,14 @@
     </row>
     <row r="16" spans="1:18" ht="14">
       <c r="A16" s="114" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B16" s="114" t="s">
+        <v>734</v>
+      </c>
+      <c r="C16" s="23"/>
+      <c r="D16" s="128" t="s">
         <v>735</v>
-      </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="131" t="s">
-        <v>736</v>
       </c>
       <c r="E16" s="23"/>
       <c r="F16" s="23"/>
@@ -13263,33 +13295,33 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:R1000"/>
+  <dimension ref="A1:R999"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="19.4140625" customWidth="1"/>
-    <col min="2" max="2" width="20.4140625" customWidth="1"/>
-    <col min="3" max="3" width="12.25" customWidth="1"/>
+    <col min="2" max="2" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.75" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.4140625" customWidth="1"/>
     <col min="5" max="21" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="14">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="146" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="146" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="46" t="s">
+      <c r="C1" s="146" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="46" t="s">
+      <c r="D1" s="146" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="62">
+      <c r="E1" s="147">
         <v>46248</v>
       </c>
-      <c r="F1" s="62">
+      <c r="F1" s="144">
         <v>46255</v>
       </c>
       <c r="G1" s="62">
@@ -13330,22 +13362,22 @@
       </c>
     </row>
     <row r="2" spans="1:18" ht="14">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="148" t="s">
         <v>682</v>
       </c>
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="148" t="s">
         <v>386</v>
       </c>
-      <c r="C2" s="51">
+      <c r="C2" s="149">
         <v>41993</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="D2" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F2" s="23"/>
+      <c r="F2" s="145"/>
       <c r="G2" s="23"/>
       <c r="H2" s="23"/>
       <c r="I2" s="23"/>
@@ -13362,22 +13394,22 @@
       <c r="R2" s="23"/>
     </row>
     <row r="3" spans="1:18" ht="14">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="148" t="s">
         <v>695</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="148" t="s">
         <v>697</v>
       </c>
-      <c r="C3" s="51">
+      <c r="C3" s="149">
         <v>42242</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F3" s="23"/>
+      <c r="F3" s="145"/>
       <c r="G3" s="23"/>
       <c r="H3" s="23"/>
       <c r="I3" s="23"/>
@@ -13394,22 +13426,22 @@
       <c r="R3" s="23"/>
     </row>
     <row r="4" spans="1:18" ht="14">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="148" t="s">
         <v>211</v>
       </c>
-      <c r="B4" s="50" t="s">
+      <c r="B4" s="148" t="s">
         <v>543</v>
       </c>
-      <c r="C4" s="51">
+      <c r="C4" s="149">
         <v>41480</v>
       </c>
-      <c r="D4" s="50" t="s">
+      <c r="D4" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F4" s="23"/>
+      <c r="F4" s="145"/>
       <c r="G4" s="23"/>
       <c r="H4" s="23"/>
       <c r="I4" s="23"/>
@@ -13426,22 +13458,22 @@
       <c r="R4" s="23"/>
     </row>
     <row r="5" spans="1:18" ht="14">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="148" t="s">
         <v>704</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="B5" s="148" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="51">
+      <c r="C5" s="149">
         <v>41190</v>
       </c>
-      <c r="D5" s="50" t="s">
+      <c r="D5" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="22" t="s">
+      <c r="E5" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F5" s="23"/>
+      <c r="F5" s="145"/>
       <c r="G5" s="23"/>
       <c r="H5" s="23"/>
       <c r="I5" s="23"/>
@@ -13458,22 +13490,22 @@
       <c r="R5" s="23"/>
     </row>
     <row r="6" spans="1:18" ht="14">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="148" t="s">
         <v>709</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="148" t="s">
         <v>357</v>
       </c>
-      <c r="C6" s="51">
+      <c r="C6" s="149">
         <v>41944</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="D6" s="148" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F6" s="23"/>
+      <c r="F6" s="145"/>
       <c r="G6" s="23"/>
       <c r="H6" s="23"/>
       <c r="I6" s="23"/>
@@ -13489,21 +13521,23 @@
       <c r="Q6" s="23"/>
       <c r="R6" s="23"/>
     </row>
-    <row r="7" spans="1:18" ht="14">
-      <c r="A7" s="128" t="s">
-        <v>602</v>
-      </c>
-      <c r="B7" s="128" t="s">
-        <v>714</v>
-      </c>
-      <c r="C7" s="51">
-        <v>41806</v>
-      </c>
-      <c r="D7" s="50" t="s">
+    <row r="7" spans="1:18" ht="15.5">
+      <c r="A7" s="151" t="s">
+        <v>715</v>
+      </c>
+      <c r="B7" s="151" t="s">
+        <v>488</v>
+      </c>
+      <c r="C7" s="152">
+        <v>41770</v>
+      </c>
+      <c r="D7" s="153" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="22"/>
-      <c r="F7" s="23"/>
+      <c r="E7" s="150" t="s">
+        <v>235</v>
+      </c>
+      <c r="F7" s="145"/>
       <c r="G7" s="23"/>
       <c r="H7" s="23"/>
       <c r="I7" s="23"/>
@@ -13519,23 +13553,23 @@
       <c r="Q7" s="23"/>
       <c r="R7" s="23"/>
     </row>
-    <row r="8" spans="1:18" ht="15.5">
-      <c r="A8" s="129" t="s">
-        <v>716</v>
-      </c>
-      <c r="B8" s="129" t="s">
-        <v>488</v>
-      </c>
-      <c r="C8" s="130">
-        <v>41770</v>
-      </c>
-      <c r="D8" s="121" t="s">
+    <row r="8" spans="1:18" ht="14">
+      <c r="A8" s="148" t="s">
+        <v>618</v>
+      </c>
+      <c r="B8" s="148" t="s">
+        <v>202</v>
+      </c>
+      <c r="C8" s="149">
+        <v>42243</v>
+      </c>
+      <c r="D8" s="153" t="s">
         <v>24</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F8" s="23"/>
+      <c r="F8" s="145"/>
       <c r="G8" s="23"/>
       <c r="H8" s="23"/>
       <c r="I8" s="23"/>
@@ -13552,22 +13586,20 @@
       <c r="R8" s="23"/>
     </row>
     <row r="9" spans="1:18" ht="14">
-      <c r="A9" s="50" t="s">
-        <v>618</v>
-      </c>
-      <c r="B9" s="50" t="s">
-        <v>202</v>
-      </c>
-      <c r="C9" s="51">
-        <v>42243</v>
-      </c>
-      <c r="D9" s="121" t="s">
+      <c r="A9" s="148" t="s">
+        <v>468</v>
+      </c>
+      <c r="B9" s="148" t="s">
+        <v>378</v>
+      </c>
+      <c r="C9" s="149"/>
+      <c r="D9" s="153" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="150" t="s">
         <v>235</v>
       </c>
-      <c r="F9" s="23"/>
+      <c r="F9" s="145"/>
       <c r="G9" s="23"/>
       <c r="H9" s="23"/>
       <c r="I9" s="23"/>
@@ -13577,106 +13609,108 @@
       <c r="M9" s="23"/>
       <c r="N9" s="23"/>
       <c r="O9" s="23"/>
-      <c r="P9" s="24" t="s">
-        <v>240</v>
-      </c>
+      <c r="P9" s="24"/>
       <c r="Q9" s="23"/>
       <c r="R9" s="23"/>
     </row>
-    <row r="10" spans="1:18" ht="14">
-      <c r="A10" s="50" t="s">
-        <v>468</v>
-      </c>
-      <c r="B10" s="50" t="s">
-        <v>378</v>
-      </c>
-      <c r="C10" s="51"/>
-      <c r="D10" s="121" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="22" t="s">
+    <row r="12" spans="1:18" ht="14">
+      <c r="A12" s="63" t="s">
+        <v>0</v>
+      </c>
+      <c r="B12" s="63" t="s">
+        <v>1</v>
+      </c>
+      <c r="C12" s="63" t="s">
+        <v>2</v>
+      </c>
+      <c r="D12" s="63" t="s">
+        <v>3</v>
+      </c>
+      <c r="E12" s="62">
+        <v>46248</v>
+      </c>
+      <c r="F12" s="62">
+        <v>46255</v>
+      </c>
+      <c r="G12" s="62">
+        <v>46262</v>
+      </c>
+      <c r="H12" s="62">
+        <v>46269</v>
+      </c>
+      <c r="I12" s="62">
+        <v>46276</v>
+      </c>
+      <c r="J12" s="62">
+        <v>46283</v>
+      </c>
+      <c r="K12" s="62">
+        <v>46290</v>
+      </c>
+      <c r="L12" s="62">
+        <v>46297</v>
+      </c>
+      <c r="M12" s="62">
+        <v>46304</v>
+      </c>
+      <c r="N12" s="64">
+        <v>46311</v>
+      </c>
+      <c r="O12" s="64">
+        <v>46318</v>
+      </c>
+      <c r="P12" s="65">
+        <v>46325</v>
+      </c>
+      <c r="Q12" s="62">
+        <v>46332</v>
+      </c>
+      <c r="R12" s="64">
+        <v>46339</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="14">
+      <c r="A13" s="69" t="s">
+        <v>548</v>
+      </c>
+      <c r="B13" s="50"/>
+      <c r="C13" s="71">
+        <v>46067</v>
+      </c>
+      <c r="D13" s="69" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="23"/>
-      <c r="R10" s="23"/>
-    </row>
-    <row r="13" spans="1:18" ht="14">
-      <c r="A13" s="63" t="s">
-        <v>0</v>
-      </c>
-      <c r="B13" s="63" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="63" t="s">
-        <v>2</v>
-      </c>
-      <c r="D13" s="63" t="s">
-        <v>3</v>
-      </c>
-      <c r="E13" s="62">
-        <v>46248</v>
-      </c>
-      <c r="F13" s="62">
-        <v>46255</v>
-      </c>
-      <c r="G13" s="62">
-        <v>46262</v>
-      </c>
-      <c r="H13" s="62">
-        <v>46269</v>
-      </c>
-      <c r="I13" s="62">
-        <v>46276</v>
-      </c>
-      <c r="J13" s="62">
-        <v>46283</v>
-      </c>
-      <c r="K13" s="62">
-        <v>46290</v>
-      </c>
-      <c r="L13" s="62">
-        <v>46297</v>
-      </c>
-      <c r="M13" s="62">
-        <v>46304</v>
-      </c>
-      <c r="N13" s="64">
-        <v>46311</v>
-      </c>
-      <c r="O13" s="64">
-        <v>46318</v>
-      </c>
-      <c r="P13" s="65">
-        <v>46325</v>
-      </c>
-      <c r="Q13" s="62">
-        <v>46332</v>
-      </c>
-      <c r="R13" s="64">
-        <v>46339</v>
-      </c>
+      <c r="F13" s="23"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="23"/>
+      <c r="P13" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q13" s="23"/>
+      <c r="R13" s="23"/>
     </row>
     <row r="14" spans="1:18" ht="14">
-      <c r="A14" s="69" t="s">
-        <v>548</v>
-      </c>
-      <c r="B14" s="50"/>
+      <c r="A14" s="114" t="s">
+        <v>146</v>
+      </c>
+      <c r="B14" s="114" t="s">
+        <v>758</v>
+      </c>
       <c r="C14" s="71">
-        <v>46067</v>
-      </c>
-      <c r="D14" s="69" t="s">
-        <v>16</v>
+        <v>46090</v>
+      </c>
+      <c r="D14" s="128" t="s">
+        <v>735</v>
       </c>
       <c r="E14" s="22" t="s">
         <v>235</v>
@@ -13697,46 +13731,15 @@
       <c r="Q14" s="23"/>
       <c r="R14" s="23"/>
     </row>
-    <row r="15" spans="1:18" ht="14">
-      <c r="A15" s="114" t="s">
-        <v>146</v>
-      </c>
-      <c r="B15" s="114" t="s">
-        <v>759</v>
-      </c>
-      <c r="C15" s="71">
-        <v>46090</v>
-      </c>
-      <c r="D15" s="131" t="s">
-        <v>736</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>235</v>
-      </c>
-      <c r="F15" s="23"/>
-      <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
-      <c r="I15" s="23"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="23"/>
-      <c r="L15" s="23"/>
-      <c r="M15" s="23"/>
-      <c r="N15" s="23"/>
-      <c r="O15" s="23"/>
-      <c r="P15" s="24" t="s">
-        <v>240</v>
-      </c>
-      <c r="Q15" s="23"/>
-      <c r="R15" s="23"/>
-    </row>
-    <row r="19" spans="1:2" ht="14">
-      <c r="A19" s="42" t="s">
+    <row r="18" spans="1:2" ht="14">
+      <c r="A18" s="42" t="s">
         <v>322</v>
       </c>
-      <c r="B19" s="42">
+      <c r="B18" s="42">
         <v>115</v>
       </c>
     </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1"/>
     <row r="21" spans="1:2" ht="15.75" customHeight="1"/>
     <row r="22" spans="1:2" ht="15.75" customHeight="1"/>
     <row r="23" spans="1:2" ht="15.75" customHeight="1"/>
@@ -14716,7 +14719,6 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -14797,12 +14799,12 @@
     </row>
     <row r="2" spans="1:19" ht="14">
       <c r="A2" s="50" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B2" s="50" t="s">
         <v>371</v>
       </c>
-      <c r="C2" s="137">
+      <c r="C2" s="134">
         <v>41688</v>
       </c>
       <c r="D2" s="50" t="s">
@@ -14832,7 +14834,7 @@
     </row>
     <row r="3" spans="1:19" ht="15.5">
       <c r="A3" s="56" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="B3" s="56" t="s">
         <v>427</v>
@@ -14840,10 +14842,10 @@
       <c r="C3" s="29">
         <v>41647</v>
       </c>
-      <c r="D3" s="138" t="s">
+      <c r="D3" s="135" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="138" t="s">
+      <c r="E3" s="135" t="s">
         <v>18</v>
       </c>
       <c r="F3" s="22" t="s">
@@ -14876,7 +14878,7 @@
         <v>2</v>
       </c>
       <c r="D6" s="63" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="E6" s="63" t="s">
         <v>3</v>
@@ -14925,8 +14927,8 @@
       </c>
     </row>
     <row r="7" spans="1:19" ht="14">
-      <c r="A7" s="139" t="s">
-        <v>747</v>
+      <c r="A7" s="136" t="s">
+        <v>746</v>
       </c>
       <c r="B7" s="67" t="s">
         <v>697</v>
@@ -14934,7 +14936,7 @@
       <c r="C7" s="68">
         <v>46193</v>
       </c>
-      <c r="D7" s="140" t="s">
+      <c r="D7" s="137" t="s">
         <v>18</v>
       </c>
       <c r="E7" s="23"/>
@@ -14950,7 +14952,7 @@
       <c r="M7" s="23"/>
       <c r="N7" s="23"/>
       <c r="O7" s="23"/>
-      <c r="P7" s="141"/>
+      <c r="P7" s="138"/>
       <c r="Q7" s="24" t="s">
         <v>240</v>
       </c>
@@ -16021,7 +16023,7 @@
     </row>
     <row r="2" spans="1:18" ht="14">
       <c r="A2" s="50" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="B2" s="50" t="s">
         <v>592</v>
@@ -16053,10 +16055,10 @@
     </row>
     <row r="3" spans="1:18" ht="14">
       <c r="A3" s="50" t="s">
+        <v>748</v>
+      </c>
+      <c r="B3" s="50" t="s">
         <v>749</v>
-      </c>
-      <c r="B3" s="50" t="s">
-        <v>750</v>
       </c>
       <c r="C3" s="51">
         <v>39779</v>
@@ -16085,7 +16087,7 @@
     </row>
     <row r="4" spans="1:18" ht="14">
       <c r="A4" s="50" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="B4" s="50" t="s">
         <v>506</v>
@@ -16117,7 +16119,7 @@
     </row>
     <row r="5" spans="1:18" ht="14">
       <c r="A5" s="50" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="B5" s="50" t="s">
         <v>246</v>
@@ -16149,7 +16151,7 @@
     </row>
     <row r="6" spans="1:18" ht="14">
       <c r="A6" s="50" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="B6" s="50" t="s">
         <v>683</v>
@@ -16181,7 +16183,7 @@
     </row>
     <row r="7" spans="1:18" ht="14">
       <c r="A7" s="50" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B7" s="50" t="s">
         <v>699</v>
@@ -16212,10 +16214,10 @@
       <c r="R7" s="23"/>
     </row>
     <row r="8" spans="1:18" ht="14.5">
-      <c r="A8" s="145" t="s">
-        <v>761</v>
-      </c>
-      <c r="B8" s="145" t="s">
+      <c r="A8" s="142" t="s">
+        <v>760</v>
+      </c>
+      <c r="B8" s="142" t="s">
         <v>548</v>
       </c>
       <c r="C8" s="51"/>
@@ -16235,7 +16237,7 @@
       <c r="M8" s="23"/>
       <c r="N8" s="23"/>
       <c r="O8" s="23"/>
-      <c r="P8" s="146" t="s">
+      <c r="P8" s="143" t="s">
         <v>240</v>
       </c>
       <c r="Q8" s="23"/>
@@ -16299,12 +16301,12 @@
     </row>
     <row r="12" spans="1:18" ht="14">
       <c r="A12" s="67" t="s">
+        <v>754</v>
+      </c>
+      <c r="B12" s="67" t="s">
         <v>755</v>
       </c>
-      <c r="B12" s="67" t="s">
-        <v>756</v>
-      </c>
-      <c r="C12" s="142">
+      <c r="C12" s="139">
         <v>46067</v>
       </c>
       <c r="D12" s="50" t="s">
@@ -16330,16 +16332,16 @@
       <c r="R12" s="23"/>
     </row>
     <row r="13" spans="1:18" ht="14">
-      <c r="A13" s="143" t="s">
-        <v>760</v>
-      </c>
-      <c r="B13" s="144" t="s">
+      <c r="A13" s="140" t="s">
+        <v>759</v>
+      </c>
+      <c r="B13" s="141" t="s">
         <v>125</v>
       </c>
-      <c r="C13" s="142">
+      <c r="C13" s="139">
         <v>46193</v>
       </c>
-      <c r="D13" s="139" t="s">
+      <c r="D13" s="136" t="s">
         <v>30</v>
       </c>
       <c r="E13" s="22" t="s">
@@ -20687,7 +20689,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="28.4140625" customWidth="1"/>
@@ -20918,7 +20920,9 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
-      <c r="A17" s="7"/>
+      <c r="A17" s="14" t="s">
+        <v>161</v>
+      </c>
       <c r="B17" s="7" t="s">
         <v>33</v>
       </c>
@@ -21052,8 +21056,8 @@
       <c r="D26" s="13"/>
     </row>
     <row r="27" spans="1:4" ht="15" customHeight="1">
-      <c r="A27" s="14" t="s">
-        <v>161</v>
+      <c r="A27" s="7" t="s">
+        <v>166</v>
       </c>
       <c r="B27" s="9" t="s">
         <v>160</v>
@@ -21061,25 +21065,15 @@
       <c r="C27" s="8"/>
       <c r="D27" s="13"/>
     </row>
-    <row r="28" spans="1:4" ht="15" customHeight="1">
+    <row r="28" spans="1:4" ht="14.5">
       <c r="A28" s="7" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B28" s="9" t="s">
         <v>160</v>
       </c>
       <c r="C28" s="8"/>
       <c r="D28" s="13"/>
-    </row>
-    <row r="29" spans="1:4" ht="14.5">
-      <c r="A29" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="C29" s="8"/>
-      <c r="D29" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21620,7 +21614,7 @@
         <v>318</v>
       </c>
       <c r="B17" s="31" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="C17" s="41" t="s">
         <v>319</v>
@@ -23154,7 +23148,7 @@
         <v>433</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="C17" s="66">
         <v>46154</v>

</xml_diff>

<commit_message>
Optimize teacher view columns, maintain attendance & homework sheets, and add Android APK package
</commit_message>
<xml_diff>
--- a/TBTA-2026-2027- RHS-Student_Attendance.xlsx
+++ b/TBTA-2026-2027- RHS-Student_Attendance.xlsx
@@ -19,6 +19,18 @@
     <sheet name="Nilai-6" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Nilai-7" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Nilai-8" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="HW_illanthalir" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="HW_Mazhalai" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="HW_Nilai-1" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="HW_Nilai-2" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="HW_Nilai-3" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="HW_Nilai-4" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="HW_Nilai-5" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="HW_Nilai-6" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="HW_Nilai-7" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="HW_Nilai-8" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Homework_Summary" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Summary_Dashboard" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FHS'!$A$1:$J$240</definedName>
@@ -18913,6 +18925,795 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Aadhavan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Kumar</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ilanthalir</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S002</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Abinaya</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Selvam</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Mazhalai</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S003</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Akilan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rajan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Amudhan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sundaram</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 2 2A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S005</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Anbarasu</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Pandian</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nilai 2 2B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S006</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Arul</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Arasan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 3 3A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S007</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Balan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Thambi</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nilai 3 3B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S008</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Chitra</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Vasagam</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 4 4A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>S009</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Devan</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Nambi</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Nilai 4 4B</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -23241,6 +24042,1235 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S010</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ezhil</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Govindan</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S011</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Iniyan</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Mani</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 6</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S012</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kailash</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Raja</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 7</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Student ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Ontime (Y/N)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Perfection (Y/N)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Handwriting (Y/N)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Effort (Y/N)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>S013</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kamali</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Kumar</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Nilai 8</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Grade / Class</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Room</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total Students</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Ontime</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Perfection</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Handwriting</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Evaluation Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ilanthalir</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mazhalai</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nilai 1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nilai 2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>122 / 125</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nilai 3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>124 / 127</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nilai 4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>129 / 130</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nilai 5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nilai 6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nilai 7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nilai 8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Grade / Class</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Room</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Total Students</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Unmarked</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Attendance Rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ilanthalir</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>126</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Mazhalai</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>116</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Nilai 1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>118</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Nilai 2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>122 / 125</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Nilai 3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>124 / 127</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nilai 4</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>129 / 130</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nilai 5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Nilai 6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>115</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Nilai 7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>117</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Nilai 8</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>111</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -24357,8 +26387,6 @@
           <t>Sundar</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
           <t>Ilanthalir (MunMazhalai)</t>

</xml_diff>